<commit_message>
Formulario para adicionar Receita / Dispesa
</commit_message>
<xml_diff>
--- a/financas_db.xlsx
+++ b/financas_db.xlsx
@@ -22,9 +22,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -64,12 +66,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -501,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -733,6 +736,40 @@
       <c r="H6" t="inlineStr">
         <is>
           <t>f73f0447</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>geovanni</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>46086</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Receita</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Salário</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>100</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Transferência</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>189d1354</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1321,7 @@
         <v>14</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>46084.7368358129</v>
+        <v>46084.73683581019</v>
       </c>
     </row>
   </sheetData>

</xml_diff>